<commit_message>
July 3 2024 changes
</commit_message>
<xml_diff>
--- a/TestData/TMTI0063927_VerifyViewCounterpartiesButtonAndViewsOnSalesforceLightningVersion.xlsx
+++ b/TestData/TMTI0063927_VerifyViewCounterpartiesButtonAndViewsOnSalesforceLightningVersion.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27726"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{403FB702-E371-4473-817F-CAEFDF6F3D80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E2E0272-5C92-4E71-A6DB-913B35E3DC4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="2" r:id="rId1"/>
@@ -176,9 +176,6 @@
     <t>A-Gas</t>
   </si>
   <si>
-    <t>Bayswater Partial Monetization</t>
-  </si>
-  <si>
     <t>View All</t>
   </si>
   <si>
@@ -342,6 +339,9 @@
   </si>
   <si>
     <t>122209-Buyers List-Tuck</t>
+  </si>
+  <si>
+    <t>Bayswater Dividend Recap</t>
   </si>
 </sst>
 </file>
@@ -729,13 +729,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -743,7 +743,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -751,12 +751,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" t="s">
         <v>47</v>
-      </c>
-      <c r="B3" t="s">
-        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -767,14 +767,14 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D30953EE-CA2E-4F7C-B9BA-21629FCB862C}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>34</v>
       </c>
@@ -782,10 +782,10 @@
         <v>39</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>41</v>
       </c>
@@ -793,10 +793,10 @@
         <v>35</v>
       </c>
       <c r="C2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>42</v>
       </c>
@@ -804,21 +804,21 @@
         <v>36</v>
       </c>
       <c r="C3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>98</v>
       </c>
       <c r="B4" t="s">
         <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -826,7 +826,7 @@
         <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -838,17 +838,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0293C6CF-D2AF-4FB5-B989-23A4E6860FD2}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -861,17 +861,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D296AE2-31EA-40C7-99FB-9B7E70535054}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -885,13 +885,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1398F625-8674-4D63-93D8-B47E3A580505}">
   <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>25</v>
       </c>
@@ -899,7 +899,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -907,10 +907,10 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B3" s="3"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="J11" s="2"/>
     </row>
   </sheetData>
@@ -922,190 +922,190 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFD13242-055E-41A8-80D8-6F50F1B57F7C}">
   <dimension ref="A1:AD2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="O1" s="7" t="s">
+      <c r="P1" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="P1" s="7" t="s">
+      <c r="Q1" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="Q1" s="7" t="s">
+      <c r="R1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="T1" s="7" t="s">
+      <c r="U1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="AD1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>79</v>
-      </c>
       <c r="B2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C2" t="s">
         <v>35</v>
       </c>
       <c r="D2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F2" t="s">
         <v>80</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
+        <v>80</v>
+      </c>
+      <c r="H2" t="s">
         <v>81</v>
       </c>
-      <c r="G2" t="s">
-        <v>81</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
+        <v>80</v>
+      </c>
+      <c r="J2" t="s">
+        <v>80</v>
+      </c>
+      <c r="K2" t="s">
         <v>82</v>
       </c>
-      <c r="I2" t="s">
-        <v>81</v>
-      </c>
-      <c r="J2" t="s">
-        <v>81</v>
-      </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>83</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>84</v>
-      </c>
-      <c r="M2" t="s">
-        <v>85</v>
       </c>
       <c r="N2" t="s">
         <v>0</v>
       </c>
       <c r="O2" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="P2" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="Q2" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="R2" t="s">
         <v>86</v>
       </c>
-      <c r="P2" s="8" t="s">
+      <c r="S2" t="s">
         <v>86</v>
       </c>
-      <c r="Q2" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="R2" t="s">
+      <c r="T2" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="S2" t="s">
-        <v>87</v>
-      </c>
-      <c r="T2" s="8" t="s">
+      <c r="U2" t="s">
         <v>88</v>
       </c>
-      <c r="U2" t="s">
+      <c r="V2" t="s">
         <v>89</v>
       </c>
-      <c r="V2" t="s">
+      <c r="W2" t="s">
         <v>90</v>
       </c>
-      <c r="W2" t="s">
+      <c r="X2" t="s">
         <v>91</v>
       </c>
-      <c r="X2" t="s">
+      <c r="Y2" t="s">
         <v>92</v>
       </c>
-      <c r="Y2" t="s">
+      <c r="Z2" t="s">
         <v>93</v>
       </c>
-      <c r="Z2" t="s">
-        <v>94</v>
-      </c>
       <c r="AA2" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AB2" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AC2" t="s">
         <v>0</v>
       </c>
       <c r="AD2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -1116,15 +1116,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6F94DFB-4724-4A5C-994B-DCCD1086734F}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="38.5703125" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="38.5546875" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.44140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -1135,7 +1135,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1146,7 +1146,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -1157,12 +1157,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C4" t="s">
         <v>97</v>
-      </c>
-      <c r="C4" t="s">
-        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -1174,14 +1174,14 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{751812A8-ABA8-4232-9D81-14F299F55479}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.5703125" customWidth="1"/>
-    <col min="3" max="3" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.5546875" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>19</v>
       </c>
@@ -1189,7 +1189,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -1205,17 +1205,17 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7552AB4B-37A5-4D47-8C03-7FFC70E2819F}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>22</v>
       </c>
@@ -1229,49 +1229,49 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBD3FF30-5810-42A4-B6D3-B7BD65EBF170}">
   <dimension ref="A1:A8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>